<commit_message>
End of June versions
</commit_message>
<xml_diff>
--- a/Use_cases/Use_case_1-Jacobsen_et_al_2024.xlsx
+++ b/Use_cases/Use_case_1-Jacobsen_et_al_2024.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://univpm-my.sharepoint.com/personal/s1116344_pm_univpm_it/Documents/PhD/ASMR/Case_studies/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\claud\Documents\COMUNE\STUDIO_LAVORO\Data_analysis\Projects\ASMR\Use_cases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="681" documentId="8_{C7C4B3F3-C924-45AD-BB41-A3CF1BA542F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{23A73CFD-E175-4113-B1B0-9837D2A9586E}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FA5D812-C8FD-4580-BF06-B110E212DC99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{C772E4A6-6938-4714-B988-E5854FC383F1}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{C772E4A6-6938-4714-B988-E5854FC383F1}"/>
   </bookViews>
   <sheets>
     <sheet name="event" sheetId="1" r:id="rId1"/>
@@ -2224,7 +2224,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -2258,7 +2258,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -3337,7 +3336,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6B605ED-3494-4570-BDCF-D71E66DDAFC5}">
-  <dimension ref="A1:W83"/>
+  <dimension ref="A1:V83"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="20.5546875" customWidth="1"/>
@@ -3629,7 +3628,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="17" spans="9:23" x14ac:dyDescent="0.3">
+    <row r="17" spans="9:22" x14ac:dyDescent="0.3">
       <c r="I17" t="s">
         <v>265</v>
       </c>
@@ -3640,7 +3639,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="18" spans="9:23" x14ac:dyDescent="0.3">
+    <row r="18" spans="9:22" x14ac:dyDescent="0.3">
       <c r="I18" s="12" t="s">
         <v>350</v>
       </c>
@@ -3654,7 +3653,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="19" spans="9:23" x14ac:dyDescent="0.3">
+    <row r="19" spans="9:22" x14ac:dyDescent="0.3">
       <c r="I19" s="12" t="s">
         <v>351</v>
       </c>
@@ -3665,7 +3664,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="20" spans="9:23" x14ac:dyDescent="0.3">
+    <row r="20" spans="9:22" x14ac:dyDescent="0.3">
       <c r="I20" t="s">
         <v>267</v>
       </c>
@@ -3676,7 +3675,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="21" spans="9:23" x14ac:dyDescent="0.3">
+    <row r="21" spans="9:22" x14ac:dyDescent="0.3">
       <c r="I21" s="12" t="s">
         <v>352</v>
       </c>
@@ -3687,99 +3686,51 @@
         <v>299</v>
       </c>
     </row>
-    <row r="22" spans="9:23" x14ac:dyDescent="0.3">
-      <c r="I22" s="13" t="s">
+    <row r="22" spans="9:22" x14ac:dyDescent="0.3">
+      <c r="I22" t="s">
         <v>269</v>
       </c>
-      <c r="J22" s="13"/>
-      <c r="K22" s="13"/>
-      <c r="L22" s="13"/>
-      <c r="M22" s="13"/>
-      <c r="N22" s="13"/>
-      <c r="O22" s="13"/>
-      <c r="P22" s="13" t="s">
+      <c r="P22" t="s">
         <v>268</v>
       </c>
-      <c r="Q22" s="13"/>
-      <c r="R22" s="13"/>
-      <c r="S22" s="13"/>
-      <c r="T22" s="13"/>
-      <c r="U22" s="13"/>
       <c r="V22" t="s">
         <v>33</v>
       </c>
-      <c r="W22" s="13"/>
-    </row>
-    <row r="23" spans="9:23" x14ac:dyDescent="0.3">
-      <c r="I23" s="13" t="s">
+    </row>
+    <row r="23" spans="9:22" x14ac:dyDescent="0.3">
+      <c r="I23" t="s">
         <v>270</v>
       </c>
-      <c r="J23" s="13"/>
-      <c r="K23" s="13"/>
-      <c r="L23" s="13"/>
-      <c r="M23" s="13"/>
-      <c r="N23" s="13"/>
-      <c r="O23" s="13"/>
-      <c r="P23" s="13" t="s">
+      <c r="P23" t="s">
         <v>268</v>
       </c>
-      <c r="Q23" s="13"/>
-      <c r="R23" s="13"/>
-      <c r="S23" s="13"/>
-      <c r="T23" s="13"/>
-      <c r="U23" s="13"/>
       <c r="V23" t="s">
         <v>33</v>
       </c>
-      <c r="W23" s="13"/>
-    </row>
-    <row r="24" spans="9:23" x14ac:dyDescent="0.3">
-      <c r="I24" s="13" t="s">
+    </row>
+    <row r="24" spans="9:22" x14ac:dyDescent="0.3">
+      <c r="I24" t="s">
         <v>271</v>
       </c>
-      <c r="J24" s="13"/>
-      <c r="K24" s="13"/>
-      <c r="L24" s="13"/>
-      <c r="M24" s="13"/>
-      <c r="N24" s="13"/>
-      <c r="O24" s="13"/>
-      <c r="P24" s="13" t="s">
+      <c r="P24" t="s">
         <v>268</v>
       </c>
-      <c r="Q24" s="13"/>
-      <c r="R24" s="13"/>
-      <c r="S24" s="13"/>
-      <c r="T24" s="13"/>
-      <c r="U24" s="13"/>
       <c r="V24" t="s">
         <v>33</v>
       </c>
-      <c r="W24" s="13"/>
-    </row>
-    <row r="25" spans="9:23" x14ac:dyDescent="0.3">
-      <c r="I25" s="13" t="s">
+    </row>
+    <row r="25" spans="9:22" x14ac:dyDescent="0.3">
+      <c r="I25" t="s">
         <v>272</v>
       </c>
-      <c r="J25" s="13"/>
-      <c r="K25" s="13"/>
-      <c r="L25" s="13"/>
-      <c r="M25" s="13"/>
-      <c r="N25" s="13"/>
-      <c r="O25" s="13"/>
-      <c r="P25" s="13" t="s">
+      <c r="P25" t="s">
         <v>268</v>
       </c>
-      <c r="Q25" s="13"/>
-      <c r="R25" s="13"/>
-      <c r="S25" s="13"/>
-      <c r="T25" s="13"/>
-      <c r="U25" s="13"/>
       <c r="V25" t="s">
         <v>33</v>
       </c>
-      <c r="W25" s="13"/>
-    </row>
-    <row r="26" spans="9:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="26" spans="9:22" x14ac:dyDescent="0.3">
       <c r="I26" t="s">
         <v>337</v>
       </c>
@@ -3790,7 +3741,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="27" spans="9:23" x14ac:dyDescent="0.3">
+    <row r="27" spans="9:22" x14ac:dyDescent="0.3">
       <c r="I27" t="s">
         <v>338</v>
       </c>
@@ -3801,7 +3752,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="28" spans="9:23" x14ac:dyDescent="0.3">
+    <row r="28" spans="9:22" x14ac:dyDescent="0.3">
       <c r="I28" t="s">
         <v>339</v>
       </c>
@@ -3812,7 +3763,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="29" spans="9:23" x14ac:dyDescent="0.3">
+    <row r="29" spans="9:22" x14ac:dyDescent="0.3">
       <c r="I29" t="s">
         <v>340</v>
       </c>
@@ -3823,7 +3774,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="30" spans="9:23" x14ac:dyDescent="0.3">
+    <row r="30" spans="9:22" x14ac:dyDescent="0.3">
       <c r="I30" t="s">
         <v>341</v>
       </c>
@@ -3834,7 +3785,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="31" spans="9:23" x14ac:dyDescent="0.3">
+    <row r="31" spans="9:22" x14ac:dyDescent="0.3">
       <c r="I31" t="s">
         <v>342</v>
       </c>
@@ -3845,7 +3796,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="32" spans="9:23" x14ac:dyDescent="0.3">
+    <row r="32" spans="9:22" x14ac:dyDescent="0.3">
       <c r="I32" t="s">
         <v>274</v>
       </c>

</xml_diff>